<commit_message>
new version of fresh project after apply design concepts
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -1447,6 +1447,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1472,6 +1475,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1491,6 +1497,1596 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId52"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId53"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId54"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId60"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId61"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId62"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId63"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId64"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId65"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId66"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId67"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId68"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId69"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="70" name="Image 70" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId70"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="71" name="Image 71" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId71"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="72" name="Image 72" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId72"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="73" name="Image 73" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId73"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="74" name="Image 74" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId74"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="75" name="Image 75" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId75"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="76" name="Image 76" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId76"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="77" name="Image 77" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId77"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="78" name="Image 78" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId78"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="79" name="Image 79" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId79"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="80" name="Image 80" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId80"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="81" name="Image 81" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId81"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="82" name="Image 82" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId82"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="83" name="Image 83" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId83"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="84" name="Image 84" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId84"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="85" name="Image 85" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId85"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="86" name="Image 86" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId86"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="87" name="Image 87" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId87"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="88" name="Image 88" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId88"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="89" name="Image 89" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId89"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="90" name="Image 90" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId90"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="91" name="Image 91" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId91"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="92" name="Image 92" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId92"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="93" name="Image 93" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId93"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="94" name="Image 94" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId94"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="95" name="Image 95" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId95"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="96" name="Image 96" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId96"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="97" name="Image 97" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId97"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="98" name="Image 98" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId98"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="99" name="Image 99" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId99"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="100" name="Image 100" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId100"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="101" name="Image 101" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId101"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="102" name="Image 102" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId102"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="103" name="Image 103" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId103"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="104" name="Image 104" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId104"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="105" name="Image 105" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId105"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1793,7 +3389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2363,6 +3959,329 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="105" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:38:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="105" customHeight="1">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:44:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="105" customHeight="1">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:47:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="105" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:52:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="105" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-06-24 09:22:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="105" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2026-06-24 09:42:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="105" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2026-06-24 09:47:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="105" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026-06-24 09:51:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="105" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:31:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="105" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:42:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="105" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:47:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="105" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:59:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="105" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:41:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="105" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-06-25 09:06:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="105" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2026-06-25 09:31:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="105" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026-06-25 10:40:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="105" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-06-25 10:44:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="105" customHeight="1">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026-06-25 10:50:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="105" customHeight="1">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:06:49</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
camera hub and ai api modulessss
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -3043,6 +3043,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3068,6 +3071,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3087,6 +3093,588 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId105"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="106" name="Image 106" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId106"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="107" name="Image 107" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId107"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="108" name="Image 108" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId108"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="109" name="Image 109" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId109"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="110" name="Image 110" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId110"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="111" name="Image 111" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId111"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="112" name="Image 112" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId112"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="113" name="Image 113" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId113"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="114" name="Image 114" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId114"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="115" name="Image 115" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId115"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="116" name="Image 116" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId116"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="117" name="Image 117" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId117"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="118" name="Image 118" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId118"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="119" name="Image 119" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId119"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="120" name="Image 120" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId120"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="121" name="Image 121" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId121"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="122" name="Image 122" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId122"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="123" name="Image 123" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId123"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="124" name="Image 124" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId124"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="125" name="Image 125" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId125"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="126" name="Image 126" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId126"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3389,7 +3977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4282,6 +4870,125 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="105" customHeight="1">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:12:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="105" customHeight="1">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:14:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="105" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-06-28 12:56:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="105" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2026-06-28 12:57:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="105" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-06-28 12:59:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="105" customHeight="1">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:02:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="105" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:03:32</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
change the IO to br var --able to change it from config file
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -3631,6 +3631,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3656,6 +3659,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3675,6 +3681,336 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId126"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="127" name="Image 127" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId127"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="128" name="Image 128" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId128"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="129" name="Image 129" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId129"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="130" name="Image 130" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId130"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="131" name="Image 131" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId131"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="132" name="Image 132" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId132"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>52</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="133" name="Image 133" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId133"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>52</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="134" name="Image 134" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId134"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>52</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="135" name="Image 135" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId135"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>53</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="136" name="Image 136" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId136"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>53</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="137" name="Image 137" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId137"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>53</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="138" name="Image 138" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId138"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3977,7 +4313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4989,6 +5325,74 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="105" customHeight="1">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:17:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="105" customHeight="1">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:29:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="105" customHeight="1">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026-06-28 15:13:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="105" customHeight="1">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-06-28 15:28:15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Cleaned up configuration and updated image formats
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +34,12 @@
       <b val="1"/>
       <color rgb="00155724"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00721C24"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +56,11 @@
         <fgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,12 +74,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -418,6 +433,734 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -720,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -759,12 +1502,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>error</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-07 10:33:17</t>
+          <t>2026-07-07 12:28:54</t>
         </is>
       </c>
     </row>
@@ -774,14 +1517,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-07 10:34:14</t>
+          <t>2026-07-07 12:30:43</t>
         </is>
       </c>
     </row>
@@ -791,14 +1534,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>pass</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-07 10:44:56</t>
+          <t>2026-07-07 12:32:18</t>
         </is>
       </c>
     </row>
@@ -808,14 +1551,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>pass</t>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-07 10:46:12</t>
+          <t>2026-07-07 13:42:14</t>
         </is>
       </c>
     </row>
@@ -825,14 +1568,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>pass</t>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-07 10:53:42</t>
+          <t>2026-07-07 13:43:47</t>
         </is>
       </c>
     </row>
@@ -842,14 +1585,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>pass</t>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-07 11:05:19</t>
+          <t>2026-07-07 13:45:19</t>
         </is>
       </c>
     </row>
@@ -859,14 +1602,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-07 11:09:10</t>
+          <t>2026-07-07 13:46:28</t>
         </is>
       </c>
     </row>
@@ -876,14 +1619,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-07 11:10:55</t>
+          <t>2026-07-07 13:47:38</t>
         </is>
       </c>
     </row>
@@ -893,14 +1636,14 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-07 11:16:25</t>
+          <t>2026-07-07 13:48:45</t>
         </is>
       </c>
     </row>
@@ -910,14 +1653,456 @@
           <t>2511TL005663ISI</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-07 11:22:23</t>
+          <t>2026-07-07 13:49:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="105" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-07-07 13:57:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="105" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-07-07 13:58:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="105" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-07-07 13:59:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="105" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:00:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="105" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:02:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="105" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:10:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="105" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:19:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="105" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:27:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="105" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:29:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="105" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:31:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="105" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:32:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="105" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:39:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="105" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:51:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="105" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:52:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="105" customHeight="1">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:55:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="105" customHeight="1">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:56:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="105" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:57:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="105" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:58:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="105" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:59:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="105" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:00:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="105" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:03:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="105" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:10:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="105" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:13:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="105" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:20:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="105" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:21:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="105" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:23:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
last version with image inhanced & full sequance
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -1161,6 +1161,118 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1463,7 +1575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2106,6 +2218,74 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="105" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-07-09 09:25:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="105" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-07-09 09:28:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="105" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-07-09 09:33:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="105" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-07-09 09:44:58</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
save last status after sequance ended
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -1273,6 +1273,90 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1575,7 +1659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2286,6 +2370,57 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="105" customHeight="1">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:10:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="105" customHeight="1">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:11:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="105" customHeight="1">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:19:03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
edit in check image status
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -1357,6 +1357,230 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1659,7 +1883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2421,6 +2645,142 @@
         </is>
       </c>
     </row>
+    <row r="45" ht="105" customHeight="1">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:23:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="105" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:24:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="105" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:26:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="105" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:30:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="105" customHeight="1">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-07-09 13:42:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="105" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-07-09 13:42:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="105" customHeight="1">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-07-09 13:45:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="105" customHeight="1">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-07-09 13:48:59</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>